<commit_message>
Update fingerprinting repository with codecFake database
</commit_message>
<xml_diff>
--- a/aucs/ljspeech/1/low_pass_filter_Avg_Spec_aucs/mahalanobis_param=1.0_nfft=128_hoplen=2_trend=False_corrtype0_1.0.xlsx
+++ b/aucs/ljspeech/1/low_pass_filter_Avg_Spec_aucs/mahalanobis_param=1.0_nfft=128_hoplen=2_trend=False_corrtype0_1.0.xlsx
@@ -438,7 +438,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.9990291941029077</v>
+        <v>0.9990297768195326</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -462,7 +462,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>0.9995175106345784</v>
+        <v>0.9995180933512033</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -478,7 +478,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>0.9970071674144864</v>
+        <v>0.9970065846978613</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -486,7 +486,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0.9945166365596411</v>
+        <v>0.9945201328593904</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -510,7 +510,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>0.9980339141075695</v>
+        <v>0.9980350795408193</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -518,7 +518,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>0.9988089272186935</v>
+        <v>0.998809451663656</v>
       </c>
     </row>
   </sheetData>
@@ -600,7 +600,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>0.9996894120389255</v>
+        <v>0.9996899947555503</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -624,7 +624,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>0.9999560048948196</v>
+        <v>0.9999560631664821</v>
       </c>
     </row>
   </sheetData>
@@ -682,7 +682,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0.99910786084727</v>
+        <v>0.999107278130645</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -690,7 +690,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>0.9993403647806072</v>
+        <v>0.9993374511974826</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -698,7 +698,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0.9934129712720704</v>
+        <v>0.9934100576889459</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -722,7 +722,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>0.9981545364489248</v>
+        <v>0.998153371015675</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -730,7 +730,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>0.998996911601888</v>
+        <v>0.9989961540702756</v>
       </c>
     </row>
   </sheetData>
@@ -812,7 +812,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.9982355340597867</v>
+        <v>0.9982349513431619</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -836,7 +836,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>0.9998235534059787</v>
+        <v>0.9998234951343162</v>
       </c>
     </row>
   </sheetData>
@@ -926,7 +926,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>0.9996940737719247</v>
+        <v>0.9996946564885496</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -942,7 +942,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>0.9999640463842433</v>
+        <v>0.9999641046559058</v>
       </c>
     </row>
   </sheetData>
@@ -1016,7 +1016,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0.98695414020162</v>
+        <v>0.9869541402016199</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1114,7 +1114,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>0.9995979255288154</v>
+        <v>0.999600256395315</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1154,7 +1154,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>0.9999431268574093</v>
+        <v>0.9999433599440593</v>
       </c>
     </row>
   </sheetData>
@@ -1220,7 +1220,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>0.9979820523279529</v>
+        <v>0.9979832177612028</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1228,7 +1228,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0.9953027212866383</v>
+        <v>0.9953038867198882</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1252,7 +1252,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>0.9954682128081115</v>
+        <v>0.9954676300914865</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -1260,7 +1260,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>0.9987196550317581</v>
+        <v>0.9987198298467456</v>
       </c>
     </row>
   </sheetData>
@@ -1294,7 +1294,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.9994598216887128</v>
+        <v>0.9994604044053377</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1366,7 +1366,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>0.9993065672163627</v>
+        <v>0.9993066254880252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>